<commit_message>
ufak: geçersiz örnekler geçerli hale getirildi
</commit_message>
<xml_diff>
--- a/docs/coklu_girdi.xlsx
+++ b/docs/coklu_girdi.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhammed.bulut\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2FFBB7-3B4A-449C-AF58-AB15311EB96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{889F9914-1576-463B-AEE9-DB237FA22000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 işe başlayanlar" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -61,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>SIRA</t>
   </si>
@@ -69,6 +80,12 @@
     <t>ATAMA OLUR TARİHİ</t>
   </si>
   <si>
+    <t>TCKN</t>
+  </si>
+  <si>
+    <t>SİCİL</t>
+  </si>
+  <si>
     <t>NOTLAR</t>
   </si>
   <si>
@@ -111,6 +128,9 @@
     <t>Sorumlu</t>
   </si>
   <si>
+    <t>CEP TEL</t>
+  </si>
+  <si>
     <t>E-POSTA HESABI</t>
   </si>
   <si>
@@ -135,29 +155,23 @@
     <t>BİRİM BELİRLEME ÇALIŞMASINDA İLK BELİRLENEN</t>
   </si>
   <si>
-    <t>SİCİL</t>
-  </si>
-  <si>
-    <t>TCKN</t>
-  </si>
-  <si>
-    <t>CEP TEL</t>
-  </si>
-  <si>
-    <t>U170</t>
-  </si>
-  <si>
-    <t>Fatma KARACA</t>
-  </si>
-  <si>
-    <t>Fatma KARA</t>
+    <t>Ayşe KOŞUK</t>
+  </si>
+  <si>
+    <t>C123</t>
+  </si>
+  <si>
+    <t>Ahsen KÜLLÜK</t>
+  </si>
+  <si>
+    <t>Z923</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -545,7 +559,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Teması">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -842,31 +856,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB137"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" customWidth="1"/>
-    <col min="10" max="10" width="21.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="10" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" customWidth="1"/>
+    <col min="10" max="10" width="21.28515625" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="14.44140625" customWidth="1"/>
-    <col min="16" max="16" width="14.88671875" customWidth="1"/>
-    <col min="18" max="19" width="18.33203125" customWidth="1"/>
-    <col min="20" max="20" width="22.88671875" customWidth="1"/>
+    <col min="15" max="15" width="14.42578125" customWidth="1"/>
+    <col min="16" max="16" width="14.85546875" customWidth="1"/>
+    <col min="18" max="19" width="18.28515625" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" customWidth="1"/>
     <col min="21" max="21" width="30" customWidth="1"/>
-    <col min="22" max="22" width="18.33203125" customWidth="1"/>
-    <col min="23" max="23" width="18.88671875" customWidth="1"/>
-    <col min="24" max="24" width="17.109375" customWidth="1"/>
-    <col min="25" max="25" width="14.33203125" customWidth="1"/>
+    <col min="22" max="22" width="18.28515625" customWidth="1"/>
+    <col min="23" max="23" width="18.85546875" customWidth="1"/>
+    <col min="24" max="24" width="17.140625" customWidth="1"/>
+    <col min="25" max="25" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" ht="70.349999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="1" customFormat="1" ht="70.349999999999994" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -874,93 +888,93 @@
         <v>1</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S1" s="4"/>
       <c r="T1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="U1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="AB1" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1">
       <c r="B2" s="8"/>
       <c r="C2" s="3">
-        <v>33755123380</v>
+        <v>58036147206</v>
       </c>
       <c r="D2" s="3">
-        <v>96697</v>
+        <v>13212</v>
       </c>
       <c r="H2" s="11"/>
       <c r="I2" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="9"/>
@@ -970,7 +984,7 @@
       <c r="O2" s="9"/>
       <c r="P2" s="9"/>
       <c r="Q2" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
@@ -978,13 +992,13 @@
       <c r="U2" s="9"/>
       <c r="Y2" s="9"/>
     </row>
-    <row r="3" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1">
       <c r="B3" s="8"/>
       <c r="C3" s="3">
-        <v>33755123380</v>
+        <v>64876364734</v>
       </c>
       <c r="D3" s="3">
-        <v>96697</v>
+        <v>32121</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="9" t="s">
@@ -998,7 +1012,7 @@
       <c r="O3" s="9"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
@@ -1006,7 +1020,7 @@
       <c r="U3" s="9"/>
       <c r="Y3" s="9"/>
     </row>
-    <row r="4" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1">
       <c r="B4" s="8"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -1026,7 +1040,7 @@
       <c r="U4" s="9"/>
       <c r="Y4" s="9"/>
     </row>
-    <row r="5" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="7" customFormat="1" ht="27.6" customHeight="1">
       <c r="B5" s="8"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -1046,7 +1060,7 @@
       <c r="U5" s="9"/>
       <c r="Y5" s="9"/>
     </row>
-    <row r="6" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="7" customFormat="1">
       <c r="B6" s="8"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -1066,7 +1080,7 @@
       <c r="U6" s="9"/>
       <c r="Y6" s="9"/>
     </row>
-    <row r="7" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="7" customFormat="1">
       <c r="B7" s="8"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -1086,7 +1100,7 @@
       <c r="U7" s="9"/>
       <c r="Y7" s="9"/>
     </row>
-    <row r="8" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="7" customFormat="1">
       <c r="B8" s="8"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -1106,7 +1120,7 @@
       <c r="U8" s="9"/>
       <c r="Y8" s="9"/>
     </row>
-    <row r="9" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="7" customFormat="1">
       <c r="B9" s="8"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -1126,7 +1140,7 @@
       <c r="U9" s="9"/>
       <c r="Y9" s="9"/>
     </row>
-    <row r="10" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="7" customFormat="1">
       <c r="B10" s="8"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -1146,7 +1160,7 @@
       <c r="U10" s="9"/>
       <c r="Y10" s="9"/>
     </row>
-    <row r="11" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="7" customFormat="1">
       <c r="B11" s="8"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -1166,7 +1180,7 @@
       <c r="U11" s="9"/>
       <c r="Y11" s="9"/>
     </row>
-    <row r="12" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="7" customFormat="1">
       <c r="B12" s="8"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -1186,7 +1200,7 @@
       <c r="U12" s="9"/>
       <c r="Y12" s="9"/>
     </row>
-    <row r="13" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="7" customFormat="1">
       <c r="B13" s="8"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -1206,7 +1220,7 @@
       <c r="U13" s="9"/>
       <c r="Y13" s="9"/>
     </row>
-    <row r="14" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="7" customFormat="1">
       <c r="B14" s="8"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1226,7 +1240,7 @@
       <c r="U14" s="9"/>
       <c r="Y14" s="9"/>
     </row>
-    <row r="15" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="7" customFormat="1">
       <c r="B15" s="8"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -1246,7 +1260,7 @@
       <c r="U15" s="9"/>
       <c r="Y15" s="9"/>
     </row>
-    <row r="16" spans="1:28" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="7" customFormat="1">
       <c r="B16" s="8"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -1266,7 +1280,7 @@
       <c r="U16" s="9"/>
       <c r="Y16" s="9"/>
     </row>
-    <row r="17" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:25" s="7" customFormat="1">
       <c r="B17" s="8"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -1286,7 +1300,7 @@
       <c r="U17" s="9"/>
       <c r="Y17" s="9"/>
     </row>
-    <row r="18" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:25" s="7" customFormat="1">
       <c r="B18" s="8"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -1306,7 +1320,7 @@
       <c r="U18" s="9"/>
       <c r="Y18" s="9"/>
     </row>
-    <row r="19" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:25" s="7" customFormat="1">
       <c r="B19" s="8"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -1326,7 +1340,7 @@
       <c r="U19" s="9"/>
       <c r="Y19" s="9"/>
     </row>
-    <row r="20" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:25" s="7" customFormat="1">
       <c r="B20" s="8"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -1346,7 +1360,7 @@
       <c r="U20" s="9"/>
       <c r="Y20" s="9"/>
     </row>
-    <row r="21" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:25" s="7" customFormat="1">
       <c r="B21" s="8"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -1366,7 +1380,7 @@
       <c r="U21" s="9"/>
       <c r="Y21" s="9"/>
     </row>
-    <row r="22" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:25" s="7" customFormat="1">
       <c r="B22" s="8"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -1386,7 +1400,7 @@
       <c r="U22" s="9"/>
       <c r="Y22" s="9"/>
     </row>
-    <row r="23" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:25" s="7" customFormat="1">
       <c r="B23" s="8"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -1406,7 +1420,7 @@
       <c r="U23" s="9"/>
       <c r="Y23" s="9"/>
     </row>
-    <row r="24" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:25" s="7" customFormat="1">
       <c r="B24" s="8"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -1426,7 +1440,7 @@
       <c r="U24" s="9"/>
       <c r="Y24" s="9"/>
     </row>
-    <row r="25" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:25" s="7" customFormat="1">
       <c r="B25" s="8"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1446,7 +1460,7 @@
       <c r="U25" s="9"/>
       <c r="Y25" s="9"/>
     </row>
-    <row r="26" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:25" s="7" customFormat="1">
       <c r="B26" s="8"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -1466,7 +1480,7 @@
       <c r="U26" s="9"/>
       <c r="Y26" s="9"/>
     </row>
-    <row r="27" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:25" s="7" customFormat="1">
       <c r="B27" s="8"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1486,7 +1500,7 @@
       <c r="U27" s="9"/>
       <c r="Y27" s="9"/>
     </row>
-    <row r="28" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:25" s="7" customFormat="1">
       <c r="B28" s="8"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1506,7 +1520,7 @@
       <c r="U28" s="9"/>
       <c r="Y28" s="9"/>
     </row>
-    <row r="29" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:25" s="7" customFormat="1">
       <c r="B29" s="8"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1526,7 +1540,7 @@
       <c r="U29" s="9"/>
       <c r="Y29" s="9"/>
     </row>
-    <row r="30" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:25" s="7" customFormat="1">
       <c r="B30" s="8"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1546,7 +1560,7 @@
       <c r="U30" s="9"/>
       <c r="Y30" s="9"/>
     </row>
-    <row r="31" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:25" s="7" customFormat="1">
       <c r="B31" s="8"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -1566,7 +1580,7 @@
       <c r="U31" s="9"/>
       <c r="Y31" s="9"/>
     </row>
-    <row r="32" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:25" s="7" customFormat="1">
       <c r="B32" s="8"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -1586,7 +1600,7 @@
       <c r="U32" s="9"/>
       <c r="Y32" s="9"/>
     </row>
-    <row r="33" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:25" s="7" customFormat="1">
       <c r="B33" s="8"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -1606,7 +1620,7 @@
       <c r="U33" s="9"/>
       <c r="Y33" s="9"/>
     </row>
-    <row r="34" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:25" s="7" customFormat="1">
       <c r="B34" s="8"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -1626,7 +1640,7 @@
       <c r="U34" s="9"/>
       <c r="Y34" s="9"/>
     </row>
-    <row r="35" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:25" s="7" customFormat="1">
       <c r="B35" s="8"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1646,7 +1660,7 @@
       <c r="U35" s="9"/>
       <c r="Y35" s="9"/>
     </row>
-    <row r="36" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:25" s="7" customFormat="1">
       <c r="B36" s="8"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -1666,7 +1680,7 @@
       <c r="U36" s="9"/>
       <c r="Y36" s="9"/>
     </row>
-    <row r="37" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:25" s="7" customFormat="1">
       <c r="B37" s="8"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -1686,7 +1700,7 @@
       <c r="U37" s="9"/>
       <c r="Y37" s="9"/>
     </row>
-    <row r="38" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:25" s="7" customFormat="1">
       <c r="B38" s="8"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -1706,7 +1720,7 @@
       <c r="U38" s="9"/>
       <c r="Y38" s="9"/>
     </row>
-    <row r="39" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:25" s="7" customFormat="1">
       <c r="B39" s="8"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -1726,7 +1740,7 @@
       <c r="U39" s="9"/>
       <c r="Y39" s="9"/>
     </row>
-    <row r="40" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:25" s="7" customFormat="1">
       <c r="B40" s="8"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -1746,7 +1760,7 @@
       <c r="U40" s="9"/>
       <c r="Y40" s="9"/>
     </row>
-    <row r="41" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:25" s="7" customFormat="1">
       <c r="B41" s="8"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -1766,292 +1780,292 @@
       <c r="U41" s="9"/>
       <c r="Y41" s="9"/>
     </row>
-    <row r="42" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:25" s="7" customFormat="1">
       <c r="B42" s="9"/>
     </row>
-    <row r="43" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:25" s="7" customFormat="1">
       <c r="B43" s="9"/>
     </row>
-    <row r="44" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:25" s="7" customFormat="1">
       <c r="B44" s="9"/>
     </row>
-    <row r="45" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:25" s="7" customFormat="1">
       <c r="B45" s="9"/>
     </row>
-    <row r="46" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:25" s="7" customFormat="1">
       <c r="B46" s="9"/>
     </row>
-    <row r="47" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:25" s="7" customFormat="1">
       <c r="B47" s="9"/>
     </row>
-    <row r="48" spans="2:25" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:25" s="7" customFormat="1">
       <c r="B48" s="9"/>
     </row>
-    <row r="49" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:2" s="7" customFormat="1">
       <c r="B49" s="9"/>
     </row>
-    <row r="50" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:2" s="7" customFormat="1">
       <c r="B50" s="9"/>
     </row>
-    <row r="51" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:2" s="7" customFormat="1">
       <c r="B51" s="9"/>
     </row>
-    <row r="52" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:2" s="7" customFormat="1">
       <c r="B52" s="9"/>
     </row>
-    <row r="53" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:2" s="7" customFormat="1">
       <c r="B53" s="9"/>
     </row>
-    <row r="54" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:2" s="7" customFormat="1">
       <c r="B54" s="9"/>
     </row>
-    <row r="55" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:2" s="7" customFormat="1">
       <c r="B55" s="9"/>
     </row>
-    <row r="56" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:2" s="7" customFormat="1">
       <c r="B56" s="9"/>
     </row>
-    <row r="57" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:2" s="7" customFormat="1">
       <c r="B57" s="9"/>
     </row>
-    <row r="58" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:2" s="7" customFormat="1">
       <c r="B58" s="9"/>
     </row>
-    <row r="59" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:2" s="7" customFormat="1">
       <c r="B59" s="9"/>
     </row>
-    <row r="60" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:2" s="7" customFormat="1">
       <c r="B60" s="9"/>
     </row>
-    <row r="61" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:2" s="7" customFormat="1">
       <c r="B61" s="9"/>
     </row>
-    <row r="62" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:2" s="7" customFormat="1">
       <c r="B62" s="9"/>
     </row>
-    <row r="63" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:2" s="7" customFormat="1">
       <c r="B63" s="9"/>
     </row>
-    <row r="64" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:2" s="7" customFormat="1">
       <c r="B64" s="9"/>
     </row>
-    <row r="65" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:2" s="7" customFormat="1">
       <c r="B65" s="9"/>
     </row>
-    <row r="66" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:2" s="7" customFormat="1">
       <c r="B66" s="9"/>
     </row>
-    <row r="67" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:2" s="7" customFormat="1">
       <c r="B67" s="9"/>
     </row>
-    <row r="68" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:2" s="7" customFormat="1">
       <c r="B68" s="9"/>
     </row>
-    <row r="69" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:2" s="7" customFormat="1">
       <c r="B69" s="9"/>
     </row>
-    <row r="70" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:2" s="7" customFormat="1">
       <c r="B70" s="9"/>
     </row>
-    <row r="71" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:2" s="7" customFormat="1">
       <c r="B71" s="9"/>
     </row>
-    <row r="72" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:2" s="7" customFormat="1">
       <c r="B72" s="9"/>
     </row>
-    <row r="73" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:2" s="7" customFormat="1">
       <c r="B73" s="9"/>
     </row>
-    <row r="74" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:2" s="7" customFormat="1">
       <c r="B74" s="9"/>
     </row>
-    <row r="75" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:2" s="7" customFormat="1">
       <c r="B75" s="9"/>
     </row>
-    <row r="76" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:2" s="7" customFormat="1">
       <c r="B76" s="9"/>
     </row>
-    <row r="77" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:2" s="7" customFormat="1">
       <c r="B77" s="9"/>
     </row>
-    <row r="78" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:2" s="7" customFormat="1">
       <c r="B78" s="9"/>
     </row>
-    <row r="79" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:2" s="7" customFormat="1">
       <c r="B79" s="9"/>
     </row>
-    <row r="80" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:2" s="7" customFormat="1">
       <c r="B80" s="9"/>
     </row>
-    <row r="81" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:2" s="7" customFormat="1">
       <c r="B81" s="9"/>
     </row>
-    <row r="82" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:2" s="7" customFormat="1">
       <c r="B82" s="9"/>
     </row>
-    <row r="83" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:2" s="7" customFormat="1">
       <c r="B83" s="9"/>
     </row>
-    <row r="84" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:2" s="7" customFormat="1">
       <c r="B84" s="9"/>
     </row>
-    <row r="85" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:2" s="7" customFormat="1">
       <c r="B85" s="9"/>
     </row>
-    <row r="86" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:2" s="7" customFormat="1">
       <c r="B86" s="9"/>
     </row>
-    <row r="87" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:2" s="7" customFormat="1">
       <c r="B87" s="9"/>
     </row>
-    <row r="88" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:2" s="7" customFormat="1">
       <c r="B88" s="9"/>
     </row>
-    <row r="89" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:2" s="7" customFormat="1">
       <c r="B89" s="9"/>
     </row>
-    <row r="90" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:2" s="7" customFormat="1">
       <c r="B90" s="9"/>
     </row>
-    <row r="91" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:2" s="7" customFormat="1">
       <c r="B91" s="9"/>
     </row>
-    <row r="92" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:2" s="7" customFormat="1">
       <c r="B92" s="9"/>
     </row>
-    <row r="93" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:2" s="7" customFormat="1">
       <c r="B93" s="9"/>
     </row>
-    <row r="94" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:2" s="7" customFormat="1">
       <c r="B94" s="9"/>
     </row>
-    <row r="95" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:2" s="7" customFormat="1">
       <c r="B95" s="9"/>
     </row>
-    <row r="96" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:2" s="7" customFormat="1">
       <c r="B96" s="9"/>
     </row>
-    <row r="97" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:2" s="7" customFormat="1">
       <c r="B97" s="9"/>
     </row>
-    <row r="98" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:2" s="7" customFormat="1">
       <c r="B98" s="9"/>
     </row>
-    <row r="99" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:2" s="7" customFormat="1">
       <c r="B99" s="9"/>
     </row>
-    <row r="100" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:2" s="7" customFormat="1">
       <c r="B100" s="9"/>
     </row>
-    <row r="101" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:2" s="7" customFormat="1">
       <c r="B101" s="9"/>
     </row>
-    <row r="102" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:2" s="7" customFormat="1">
       <c r="B102" s="9"/>
     </row>
-    <row r="103" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:2" s="7" customFormat="1">
       <c r="B103" s="9"/>
     </row>
-    <row r="104" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:2" s="7" customFormat="1">
       <c r="B104" s="9"/>
     </row>
-    <row r="105" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:2" s="7" customFormat="1">
       <c r="B105" s="9"/>
     </row>
-    <row r="106" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:2" s="7" customFormat="1">
       <c r="B106" s="9"/>
     </row>
-    <row r="107" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:2" s="7" customFormat="1">
       <c r="B107" s="9"/>
     </row>
-    <row r="108" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:2" s="7" customFormat="1">
       <c r="B108" s="9"/>
     </row>
-    <row r="109" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:2" s="7" customFormat="1">
       <c r="B109" s="9"/>
     </row>
-    <row r="110" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:2" s="7" customFormat="1">
       <c r="B110" s="9"/>
     </row>
-    <row r="111" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:2" s="7" customFormat="1">
       <c r="B111" s="9"/>
     </row>
-    <row r="112" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:2" s="7" customFormat="1">
       <c r="B112" s="9"/>
     </row>
-    <row r="113" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:2" s="7" customFormat="1">
       <c r="B113" s="9"/>
     </row>
-    <row r="114" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:2" s="7" customFormat="1">
       <c r="B114" s="9"/>
     </row>
-    <row r="115" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:2" s="7" customFormat="1">
       <c r="B115" s="9"/>
     </row>
-    <row r="116" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:2" s="7" customFormat="1">
       <c r="B116" s="9"/>
     </row>
-    <row r="117" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:2" s="7" customFormat="1">
       <c r="B117" s="9"/>
     </row>
-    <row r="118" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:2" s="7" customFormat="1">
       <c r="B118" s="9"/>
     </row>
-    <row r="119" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:2" s="7" customFormat="1">
       <c r="B119" s="9"/>
     </row>
-    <row r="120" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:2" s="7" customFormat="1">
       <c r="B120" s="9"/>
     </row>
-    <row r="121" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:2" s="7" customFormat="1">
       <c r="B121" s="9"/>
     </row>
-    <row r="122" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:2" s="7" customFormat="1">
       <c r="B122" s="9"/>
     </row>
-    <row r="123" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:2" s="7" customFormat="1">
       <c r="B123" s="9"/>
     </row>
-    <row r="124" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:2" s="7" customFormat="1">
       <c r="B124" s="9"/>
     </row>
-    <row r="125" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:2" s="7" customFormat="1">
       <c r="B125" s="9"/>
     </row>
-    <row r="126" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:2" s="7" customFormat="1">
       <c r="B126" s="9"/>
     </row>
-    <row r="127" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:2" s="7" customFormat="1">
       <c r="B127" s="9"/>
     </row>
-    <row r="128" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:2" s="7" customFormat="1">
       <c r="B128" s="9"/>
     </row>
-    <row r="129" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:2" s="7" customFormat="1">
       <c r="B129" s="9"/>
     </row>
-    <row r="130" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:2" s="7" customFormat="1">
       <c r="B130" s="9"/>
     </row>
-    <row r="131" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:2" s="7" customFormat="1">
       <c r="B131" s="9"/>
     </row>
-    <row r="132" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:2" s="7" customFormat="1">
       <c r="B132" s="9"/>
     </row>
-    <row r="133" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:2" s="7" customFormat="1">
       <c r="B133" s="9"/>
     </row>
-    <row r="134" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:2" s="7" customFormat="1">
       <c r="B134" s="9"/>
     </row>
-    <row r="135" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:2" s="7" customFormat="1">
       <c r="B135" s="9"/>
     </row>
-    <row r="136" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:2" s="7" customFormat="1">
       <c r="B136" s="9"/>
     </row>
-    <row r="137" spans="2:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:2" s="7" customFormat="1">
       <c r="B137" s="9"/>
     </row>
   </sheetData>

</xml_diff>